<commit_message>
Botao Consultar nas telas em que o registro travava depois de finalizado
Titulo baixado, ordem de producao ja iniciada e falta ja abonada nao
podem mais ser editados -- e, sem botao nenhum, tambem nao podiam ser
abertos. Ganham um botao de olho sempre disponivel que abre o mesmo
formulario travado: os campos ficam num fieldset disabled (trava tudo de
uma vez, sem repetir condicao em cada campo) e o rodape mostra so
Fechar, sem Salvar

Vale pra contas a pagar e a receber, ordens de producao e faltas. As
telas de documento (pedidos, orcamentos, cotacoes, vendas, compras,
folha, ferias e 13o) ja tinham o olho de "Ver itens" disponivel em
qualquer situacao
</commit_message>
<xml_diff>
--- a/docs/planos.xlsx
+++ b/docs/planos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projeto\SaaS\AlePejoERP\alepejo-erp-cloud\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D5AFD90-BF5B-4A2C-A0D2-96F9E0987AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49710A4-D902-44C1-984F-AB827E30E65F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-5865" windowWidth="16440" windowHeight="28320" xr2:uid="{A80D30AC-C001-49B4-9C21-A5AA2258F82D}"/>
   </bookViews>
@@ -429,13 +429,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ED632B9-1B15-420F-AFC5-5A4AE6CDE114}">
   <sheetPr codeName="Folha1"/>
-  <dimension ref="B4:I24"/>
+  <dimension ref="B4:M24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>129.9</v>
       </c>
@@ -444,33 +444,33 @@
         <v>1558.8000000000002</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C5">
         <v>300</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="C6">
         <f>C4-C5</f>
         <v>1258.8000000000002</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>3</v>
       </c>
@@ -478,35 +478,47 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>4</v>
       </c>
       <c r="C15">
-        <v>59.9</v>
+        <v>79.900000000000006</v>
       </c>
       <c r="D15">
         <f>C15*12</f>
-        <v>718.8</v>
+        <v>958.80000000000007</v>
       </c>
       <c r="E15">
         <f>D15*0.85</f>
-        <v>610.9799999999999</v>
+        <v>814.98</v>
       </c>
       <c r="F15">
         <f>D15-E15</f>
-        <v>107.82000000000005</v>
+        <v>143.82000000000005</v>
       </c>
       <c r="H15">
         <f>C15</f>
-        <v>59.9</v>
+        <v>79.900000000000006</v>
       </c>
       <c r="I15">
         <f>E15</f>
-        <v>610.9799999999999</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+        <v>814.98</v>
+      </c>
+      <c r="K15">
+        <f>H15*10</f>
+        <v>799</v>
+      </c>
+      <c r="L15">
+        <f>H15*100</f>
+        <v>7990.0000000000009</v>
+      </c>
+      <c r="M15">
+        <f>H15*300</f>
+        <v>23970</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>5</v>
       </c>
@@ -570,11 +582,11 @@
       </c>
       <c r="H18">
         <f>C15+C16</f>
-        <v>80.8</v>
+        <v>100.80000000000001</v>
       </c>
       <c r="I18">
         <f>E15+E16</f>
-        <v>824.15999999999985</v>
+        <v>1028.1600000000001</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
@@ -623,27 +635,27 @@
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="C21">
         <f>SUM(C15:C20)</f>
-        <v>153.4</v>
+        <v>173.40000000000003</v>
       </c>
       <c r="D21">
         <f>SUM(D15:D20)</f>
-        <v>1840.7999999999997</v>
+        <v>2080.8000000000002</v>
       </c>
       <c r="E21">
         <f t="shared" si="1"/>
-        <v>1564.6799999999998</v>
+        <v>1768.68</v>
       </c>
       <c r="F21">
         <f t="shared" si="2"/>
-        <v>276.11999999999989</v>
+        <v>312.12000000000012</v>
       </c>
       <c r="H21">
         <f>C15+C16+C18+C17</f>
-        <v>113.6</v>
+        <v>133.60000000000002</v>
       </c>
       <c r="I21">
-        <f>E18+E19</f>
-        <v>334.55999999999995</v>
+        <f>E15+E16+E18+E17</f>
+        <v>1362.72</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
@@ -654,11 +666,11 @@
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H24">
         <f>C21</f>
-        <v>153.4</v>
+        <v>173.40000000000003</v>
       </c>
       <c r="I24">
-        <f>E21+E22</f>
-        <v>1564.6799999999998</v>
+        <f>E21</f>
+        <v>1768.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Amplia limite de listagem para relatorios; separa permissoes de Importar/Exportar Parceiros; botao Limpar tudo nas notificacoes
- Filtros de listagem (Parceiros, Produtos, Estoque, Financeiro, RH etc.) passam de 20/100 para 10000 registros, permitindo que os relatorios tragam a base inteira.
- Nova permissao "partner.import" e "partner.export", desacopladas de "partner.create" - matriz de Perfis ganha colunas proprias e script de backfill concede ao perfil Administrador existente.
- Sino de notificacoes ganha botao "Limpar tudo" (marcar todas como lidas de uma vez).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018GpvNeiVydzyiXFvwrniXU
</commit_message>
<xml_diff>
--- a/docs/planos.xlsx
+++ b/docs/planos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projeto\SaaS\AlePejoERP\alepejo-erp-cloud\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D49710A4-D902-44C1-984F-AB827E30E65F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{399895C7-FA7A-4B6B-AA02-D5852E43AE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-5865" windowWidth="16440" windowHeight="28320" xr2:uid="{A80D30AC-C001-49B4-9C21-A5AA2258F82D}"/>
   </bookViews>
@@ -83,7 +83,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,14 +119,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Vírgula" xfId="1" builtinId="3"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -429,7 +442,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1ED632B9-1B15-420F-AFC5-5A4AE6CDE114}">
   <sheetPr codeName="Folha1"/>
-  <dimension ref="B4:M24"/>
+  <dimension ref="B4:M30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
@@ -459,21 +472,81 @@
       <c r="B11" t="s">
         <v>0</v>
       </c>
+      <c r="C11" s="1">
+        <v>2.9</v>
+      </c>
+      <c r="D11">
+        <f t="shared" ref="D11:D14" si="0">C11*12</f>
+        <v>34.799999999999997</v>
+      </c>
+      <c r="E11">
+        <f t="shared" ref="E11:E14" si="1">D11*0.85</f>
+        <v>29.58</v>
+      </c>
+      <c r="F11">
+        <f t="shared" ref="F11:F14" si="2">D11-E11</f>
+        <v>5.2199999999999989</v>
+      </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>1</v>
       </c>
+      <c r="C12" s="1">
+        <v>2.9</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>34.799999999999997</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>29.58</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="2"/>
+        <v>5.2199999999999989</v>
+      </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>2</v>
       </c>
+      <c r="C13" s="1">
+        <v>10.9</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>130.80000000000001</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="1"/>
+        <v>111.18</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="2"/>
+        <v>19.620000000000005</v>
+      </c>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>3</v>
       </c>
+      <c r="C14" s="1">
+        <v>10.9</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="0"/>
+        <v>130.80000000000001</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="1"/>
+        <v>111.18</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="2"/>
+        <v>19.620000000000005</v>
+      </c>
       <c r="H14" t="s">
         <v>10</v>
       </c>
@@ -482,80 +555,80 @@
       <c r="B15" t="s">
         <v>4</v>
       </c>
-      <c r="C15">
-        <v>79.900000000000006</v>
+      <c r="C15" s="1">
+        <v>10.9</v>
       </c>
       <c r="D15">
         <f>C15*12</f>
-        <v>958.80000000000007</v>
+        <v>130.80000000000001</v>
       </c>
       <c r="E15">
         <f>D15*0.85</f>
-        <v>814.98</v>
+        <v>111.18</v>
       </c>
       <c r="F15">
         <f>D15-E15</f>
-        <v>143.82000000000005</v>
+        <v>19.620000000000005</v>
       </c>
       <c r="H15">
         <f>C15</f>
-        <v>79.900000000000006</v>
+        <v>10.9</v>
       </c>
       <c r="I15">
         <f>E15</f>
-        <v>814.98</v>
+        <v>111.18</v>
       </c>
       <c r="K15">
         <f>H15*10</f>
-        <v>799</v>
+        <v>109</v>
       </c>
       <c r="L15">
         <f>H15*100</f>
-        <v>7990.0000000000009</v>
+        <v>1090</v>
       </c>
       <c r="M15">
         <f>H15*300</f>
-        <v>23970</v>
+        <v>3270</v>
       </c>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>5</v>
       </c>
-      <c r="C16">
-        <v>20.9</v>
+      <c r="C16" s="1">
+        <v>29.9</v>
       </c>
       <c r="D16">
-        <f t="shared" ref="D16:D20" si="0">C16*12</f>
-        <v>250.79999999999998</v>
+        <f t="shared" ref="D16:D22" si="3">C16*12</f>
+        <v>358.79999999999995</v>
       </c>
       <c r="E16">
-        <f t="shared" ref="E16:E21" si="1">D16*0.85</f>
-        <v>213.17999999999998</v>
+        <f t="shared" ref="E16:E21" si="4">D16*0.85</f>
+        <v>304.97999999999996</v>
       </c>
       <c r="F16">
-        <f t="shared" ref="F16:F21" si="2">D16-E16</f>
-        <v>37.620000000000005</v>
+        <f t="shared" ref="F16:F21" si="5">D16-E16</f>
+        <v>53.819999999999993</v>
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>6</v>
       </c>
-      <c r="C17">
-        <v>9.9</v>
+      <c r="C17" s="1">
+        <v>3.9</v>
       </c>
       <c r="D17">
-        <f t="shared" si="0"/>
-        <v>118.80000000000001</v>
+        <f t="shared" si="3"/>
+        <v>46.8</v>
       </c>
       <c r="E17">
-        <f t="shared" si="1"/>
-        <v>100.98</v>
+        <f t="shared" si="4"/>
+        <v>39.779999999999994</v>
       </c>
       <c r="F17">
-        <f t="shared" si="2"/>
-        <v>17.820000000000007</v>
+        <f t="shared" si="5"/>
+        <v>7.0200000000000031</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
@@ -565,47 +638,47 @@
       <c r="B18" t="s">
         <v>7</v>
       </c>
-      <c r="C18">
-        <v>22.9</v>
+      <c r="C18" s="1">
+        <v>33.9</v>
       </c>
       <c r="D18">
-        <f t="shared" si="0"/>
-        <v>274.79999999999995</v>
+        <f t="shared" si="3"/>
+        <v>406.79999999999995</v>
       </c>
       <c r="E18">
-        <f t="shared" si="1"/>
-        <v>233.57999999999996</v>
+        <f t="shared" si="4"/>
+        <v>345.78</v>
       </c>
       <c r="F18">
-        <f t="shared" si="2"/>
-        <v>41.22</v>
+        <f t="shared" si="5"/>
+        <v>61.019999999999982</v>
       </c>
       <c r="H18">
         <f>C15+C16</f>
-        <v>100.80000000000001</v>
+        <v>40.799999999999997</v>
       </c>
       <c r="I18">
         <f>E15+E16</f>
-        <v>1028.1600000000001</v>
+        <v>416.15999999999997</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>8</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="1">
         <v>9.9</v>
       </c>
       <c r="D19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>118.80000000000001</v>
       </c>
       <c r="E19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>100.98</v>
       </c>
       <c r="F19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>17.820000000000007</v>
       </c>
     </row>
@@ -613,49 +686,49 @@
       <c r="B20" t="s">
         <v>9</v>
       </c>
-      <c r="C20">
-        <v>29.9</v>
+      <c r="C20" s="1">
+        <v>33.9</v>
       </c>
       <c r="D20">
-        <f t="shared" si="0"/>
-        <v>358.79999999999995</v>
+        <f t="shared" si="3"/>
+        <v>406.79999999999995</v>
       </c>
       <c r="E20">
-        <f t="shared" si="1"/>
-        <v>304.97999999999996</v>
+        <f t="shared" si="4"/>
+        <v>345.78</v>
       </c>
       <c r="F20">
-        <f t="shared" si="2"/>
-        <v>53.819999999999993</v>
+        <f t="shared" si="5"/>
+        <v>61.019999999999982</v>
       </c>
       <c r="H20" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C21">
-        <f>SUM(C15:C20)</f>
-        <v>173.40000000000003</v>
+      <c r="C21" s="1">
+        <f>SUM(C11:C20)</f>
+        <v>150.00000000000003</v>
       </c>
       <c r="D21">
         <f>SUM(D15:D20)</f>
-        <v>2080.8000000000002</v>
+        <v>1468.8</v>
       </c>
       <c r="E21">
-        <f t="shared" si="1"/>
-        <v>1768.68</v>
+        <f t="shared" si="4"/>
+        <v>1248.48</v>
       </c>
       <c r="F21">
-        <f t="shared" si="2"/>
-        <v>312.12000000000012</v>
+        <f t="shared" si="5"/>
+        <v>220.31999999999994</v>
       </c>
       <c r="H21">
         <f>C15+C16+C18+C17</f>
-        <v>133.60000000000002</v>
+        <v>78.599999999999994</v>
       </c>
       <c r="I21">
         <f>E15+E16+E18+E17</f>
-        <v>1362.72</v>
+        <v>801.71999999999991</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
@@ -666,11 +739,30 @@
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H24">
         <f>C21</f>
-        <v>173.40000000000003</v>
+        <v>150.00000000000003</v>
       </c>
       <c r="I24">
         <f>E21</f>
-        <v>1768.68</v>
+        <v>1248.48</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C28" s="1">
+        <v>89.9</v>
+      </c>
+      <c r="D28">
+        <f>C28*12</f>
+        <v>1078.8000000000002</v>
+      </c>
+      <c r="E28">
+        <f t="shared" ref="E28" si="6">D28*0.85</f>
+        <v>916.98000000000013</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C30">
+        <f>C29/5</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>